<commit_message>
Update dataset type name to "Whole Exome Sequencing (WES)"
</commit_message>
<xml_diff>
--- a/wes/latest/wes.xlsx
+++ b/wes/latest/wes.xlsx
@@ -361,7 +361,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="809">
   <si>
     <t>parent_sample_id</t>
   </si>
@@ -729,2046 +729,2049 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000504</t>
   </si>
   <si>
+    <t>Whole Exome Sequencing (WES)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000514</t>
+  </si>
+  <si>
+    <t>analyte_class</t>
+  </si>
+  <si>
+    <t>Chromatin</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C13201</t>
+  </si>
+  <si>
+    <t>Collagen</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C16447</t>
+  </si>
+  <si>
+    <t>Protein</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17021</t>
+  </si>
+  <si>
+    <t>DNA</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C449</t>
+  </si>
+  <si>
+    <t>Metabolite</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C61154</t>
+  </si>
+  <si>
+    <t>Lipid</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C616</t>
+  </si>
+  <si>
+    <t>Peptide</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C735</t>
+  </si>
+  <si>
+    <t>RNA</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C812</t>
+  </si>
+  <si>
+    <t>Polysaccharide</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_18154</t>
+  </si>
+  <si>
+    <t>Fluorochrome</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/CHEBI_51217</t>
+  </si>
+  <si>
+    <t>Endogenous fluorophore</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000131</t>
+  </si>
+  <si>
+    <t>Nucleic acid + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000273</t>
+  </si>
+  <si>
+    <t>DNA + RNA</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000327</t>
+  </si>
+  <si>
+    <t>Saturated lipid</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000388</t>
+  </si>
+  <si>
+    <t>Unsaturated lipid</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000389</t>
+  </si>
+  <si>
+    <t>Lipid + metabolite</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000401</t>
+  </si>
+  <si>
+    <t>RNA + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000474</t>
+  </si>
+  <si>
+    <t>Lipid + metabolite + protein</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000478</t>
+  </si>
+  <si>
+    <t>is_targeted</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>acquisition_instrument_vendor</t>
+  </si>
+  <si>
+    <t>In-House</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C126386</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_003899</t>
+  </si>
+  <si>
+    <t>Thermo Fisher Scientific</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008452</t>
+  </si>
+  <si>
+    <t>Leica Microsystems</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008960</t>
+  </si>
+  <si>
+    <t>Miltenyi Biotec</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008984</t>
+  </si>
+  <si>
+    <t>Illumina</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_010233</t>
+  </si>
+  <si>
+    <t>Hamamatsu</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017105</t>
+  </si>
+  <si>
+    <t>Bruker</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017365</t>
+  </si>
+  <si>
+    <t>Cytiva</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023581</t>
+  </si>
+  <si>
+    <t>Leica Biosystems</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023603</t>
+  </si>
+  <si>
+    <t>Keyence</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023604</t>
+  </si>
+  <si>
+    <t>Ionpath</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023605</t>
+  </si>
+  <si>
+    <t>Standard BioTools (Fluidigm)</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023606</t>
+  </si>
+  <si>
+    <t>Zeiss Microscopy</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023607</t>
+  </si>
+  <si>
+    <t>Andor</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023609</t>
+  </si>
+  <si>
+    <t>Sciex</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023651</t>
+  </si>
+  <si>
+    <t>10x Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023672</t>
+  </si>
+  <si>
+    <t>Akoya Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023774</t>
+  </si>
+  <si>
+    <t>Resolve Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023911</t>
+  </si>
+  <si>
+    <t>NanoString</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023912</t>
+  </si>
+  <si>
+    <t>Waters</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024589</t>
+  </si>
+  <si>
+    <t>Evident Scientific (Olympus)</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024782</t>
+  </si>
+  <si>
+    <t>BGI Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024848</t>
+  </si>
+  <si>
+    <t>Motic</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024856</t>
+  </si>
+  <si>
+    <t>Huron Digital Pathology</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024996</t>
+  </si>
+  <si>
+    <t>GE Healthcare</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025461</t>
+  </si>
+  <si>
+    <t>Vizgen</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026274</t>
+  </si>
+  <si>
+    <t>Element Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026453</t>
+  </si>
+  <si>
+    <t>Singular Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026683</t>
+  </si>
+  <si>
+    <t>Complete Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027007</t>
+  </si>
+  <si>
+    <t>3DHISTECH</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027042</t>
+  </si>
+  <si>
+    <t>Cytek Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027071</t>
+  </si>
+  <si>
+    <t>Microscopes International</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027094</t>
+  </si>
+  <si>
+    <t>Revvity</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027779</t>
+  </si>
+  <si>
+    <t>MGI Tech</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_029020</t>
+  </si>
+  <si>
+    <t>acquisition_instrument_model</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17998</t>
+  </si>
+  <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C48660</t>
+  </si>
+  <si>
+    <t>NextSeq 500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_014983</t>
+  </si>
+  <si>
+    <t>NextSeq 550</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016381</t>
+  </si>
+  <si>
+    <t>HiSeq 2500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016383</t>
+  </si>
+  <si>
+    <t>HiSeq 4000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016386</t>
+  </si>
+  <si>
+    <t>NovaSeq 6000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016387</t>
+  </si>
+  <si>
+    <t>iScan System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_016388</t>
+  </si>
+  <si>
+    <t>BZ-X710</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017202</t>
+  </si>
+  <si>
+    <t>LSM 710 Confocal Microscope</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_018063</t>
+  </si>
+  <si>
+    <t>Helios</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_019916</t>
+  </si>
+  <si>
+    <t>QTRAP 5500</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020517</t>
+  </si>
+  <si>
+    <t>Q Exactive HF</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020558</t>
+  </si>
+  <si>
+    <t>Orbitrap Fusion Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020559</t>
+  </si>
+  <si>
+    <t>Orbitrap Fusion Lumos Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020562</t>
+  </si>
+  <si>
+    <t>Q Exactive HF-X</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020564</t>
+  </si>
+  <si>
+    <t>Q Exactive</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020565</t>
+  </si>
+  <si>
+    <t>Q Exactive UHMR</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020571</t>
+  </si>
+  <si>
+    <t>Zeiss LightSheet Z.1</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020919</t>
+  </si>
+  <si>
+    <t>Axio Scan.Z1</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_020927</t>
+  </si>
+  <si>
+    <t>Aperio AT2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021256</t>
+  </si>
+  <si>
+    <t>NanoZoomer 2.0-HT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021658</t>
+  </si>
+  <si>
+    <t>Digital Spatial Profiler</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_021660</t>
+  </si>
+  <si>
+    <t>Biomark HD</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_022658</t>
+  </si>
+  <si>
+    <t>Hyperion Imaging System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023195</t>
+  </si>
+  <si>
+    <t>PhenoImager Fusion</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023274</t>
+  </si>
+  <si>
+    <t>Zyla 4.2 sCMOS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023610</t>
+  </si>
+  <si>
+    <t>SCN400</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023611</t>
+  </si>
+  <si>
+    <t>MIBIscope</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023613</t>
+  </si>
+  <si>
+    <t>NextSeq 2000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023614</t>
+  </si>
+  <si>
+    <t>timsTOF FleX MALDI-2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023615</t>
+  </si>
+  <si>
+    <t>IN Cell Analyzer 2200</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023616</t>
+  </si>
+  <si>
+    <t>BZ-X800</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023617</t>
+  </si>
+  <si>
+    <t>Orbitrap Eclipse Tribrid</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023618</t>
+  </si>
+  <si>
+    <t>Axio Observer 5</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023692</t>
+  </si>
+  <si>
+    <t>Axio Observer 3</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023693</t>
+  </si>
+  <si>
+    <t>Axio Observer 7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023694</t>
+  </si>
+  <si>
+    <t>NanoZoomer S210</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023760</t>
+  </si>
+  <si>
+    <t>NanoZoomer S360</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023761</t>
+  </si>
+  <si>
+    <t>NanoZoomer S60</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023762</t>
+  </si>
+  <si>
+    <t>NanoZoomer-SQ</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023763</t>
+  </si>
+  <si>
+    <t>Phenocycler-Fusion 2.0</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023773</t>
+  </si>
+  <si>
+    <t>CosMx Spatial Molecular Imager</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023909</t>
+  </si>
+  <si>
+    <t>Xenium Analyzer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023910</t>
+  </si>
+  <si>
+    <t>Lightsheet 7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024448</t>
+  </si>
+  <si>
+    <t>Resolve Biosciences Molecular Cartography</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024449</t>
+  </si>
+  <si>
+    <t>NovaSeq X Plus</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024568</t>
+  </si>
+  <si>
+    <t>NovaSeq X</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024569</t>
+  </si>
+  <si>
+    <t>STELLARIS 5</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024663</t>
+  </si>
+  <si>
+    <t>VS200 Slide Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024783</t>
+  </si>
+  <si>
+    <t>Pannoramic MIDI II Digital Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024834</t>
+  </si>
+  <si>
+    <t>DNBSEQ-T7</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024847</t>
+  </si>
+  <si>
+    <t>MoticEasyScan One</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024855</t>
+  </si>
+  <si>
+    <t>DM6 B</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024857</t>
+  </si>
+  <si>
+    <t>TissueScope LE Slide Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024995</t>
+  </si>
+  <si>
+    <t>EVOS M7000</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025070</t>
+  </si>
+  <si>
+    <t>Aperio CS2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025111</t>
+  </si>
+  <si>
+    <t>BZ-X810</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025160</t>
+  </si>
+  <si>
+    <t>MERSCOPE Ultra</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026273</t>
+  </si>
+  <si>
+    <t>CyTOF XT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026344</t>
+  </si>
+  <si>
+    <t>AVITI24</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026452</t>
+  </si>
+  <si>
+    <t>SYNAPT XS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026524</t>
+  </si>
+  <si>
+    <t>timsTOF Ultra</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026540</t>
+  </si>
+  <si>
+    <t>timsTOF Ultra 2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026541</t>
+  </si>
+  <si>
+    <t>timsTOF SCP</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026542</t>
+  </si>
+  <si>
+    <t>timsTOF HT</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026543</t>
+  </si>
+  <si>
+    <t>timsTOF Pro</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026544</t>
+  </si>
+  <si>
+    <t>timsTOF Pro 2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026545</t>
+  </si>
+  <si>
+    <t>CyTOF 2</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026551</t>
+  </si>
+  <si>
+    <t>DMi8</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026672</t>
+  </si>
+  <si>
+    <t>G4X Spatial Sequencer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026684</t>
+  </si>
+  <si>
+    <t>timsTOF FleX</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_026925</t>
+  </si>
+  <si>
+    <t>Cytek Northern Lights</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027072</t>
+  </si>
+  <si>
+    <t>Axio Zoom.V16</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027090</t>
+  </si>
+  <si>
+    <t>solariX</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027095</t>
+  </si>
+  <si>
+    <t>uScopeHXII-20</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027101</t>
+  </si>
+  <si>
+    <t>Juno System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027198</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027323</t>
+  </si>
+  <si>
+    <t>Panoramic 150 Digital Scanner</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027467</t>
+  </si>
+  <si>
+    <t>Opera Phenix Plus HCS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027780</t>
+  </si>
+  <si>
+    <t>SYNAPT G2-Si</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027782</t>
+  </si>
+  <si>
+    <t>Opera Phenix HCS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027817</t>
+  </si>
+  <si>
+    <t>MACSima System</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_027923</t>
+  </si>
+  <si>
+    <t>NanoZoomer 2.0-RS</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_028001</t>
+  </si>
+  <si>
+    <t>Orbitrap Astral</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_028684</t>
+  </si>
+  <si>
+    <t>Olink Signature Q100</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_028906</t>
+  </si>
+  <si>
+    <t>Phenocycler-Fusion 1.0</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000316</t>
+  </si>
+  <si>
+    <t>Custom: Multiphoton</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000317</t>
+  </si>
+  <si>
+    <t>MERSCOPE</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000404</t>
+  </si>
+  <si>
+    <t>MALDI timsTOF Flex Prototype</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000433</t>
+  </si>
+  <si>
+    <t>source_storage_duration_value</t>
+  </si>
+  <si>
+    <t>source_storage_duration_unit</t>
+  </si>
+  <si>
+    <t>minute</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000031</t>
+  </si>
+  <si>
+    <t>hour</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000032</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000033</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000035</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000036</t>
+  </si>
+  <si>
+    <t>time_since_acquisition_instrument_calibration_value</t>
+  </si>
+  <si>
+    <t>time_since_acquisition_instrument_calibration_unit</t>
+  </si>
+  <si>
+    <t>contributors_path</t>
+  </si>
+  <si>
+    <t>data_path</t>
+  </si>
+  <si>
+    <t>assay_input_entity</t>
+  </si>
+  <si>
+    <t>tissue (bulk)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000267</t>
+  </si>
+  <si>
+    <t>single cell</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000268</t>
+  </si>
+  <si>
+    <t>single nucleus</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000269</t>
+  </si>
+  <si>
+    <t>spot</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000270</t>
+  </si>
+  <si>
+    <t>area of interest</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000271</t>
+  </si>
+  <si>
+    <t>amount_of_input_analyte_value</t>
+  </si>
+  <si>
+    <t>amount_of_input_analyte_unit</t>
+  </si>
+  <si>
+    <t>ug</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000023</t>
+  </si>
+  <si>
+    <t>ng</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000024</t>
+  </si>
+  <si>
+    <t>library_adapter_sequence</t>
+  </si>
+  <si>
+    <t>library_average_fragment_size</t>
+  </si>
+  <si>
+    <t>dna_assay_input_value</t>
+  </si>
+  <si>
+    <t>dna_assay_input_unit</t>
+  </si>
+  <si>
+    <t>library_output_amount_value</t>
+  </si>
+  <si>
+    <t>library_output_amount_unit</t>
+  </si>
+  <si>
+    <t>ul</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000101</t>
+  </si>
+  <si>
+    <t>library_concentration_value</t>
+  </si>
+  <si>
+    <t>library_concentration_unit</t>
+  </si>
+  <si>
+    <t>nM</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0000065</t>
+  </si>
+  <si>
+    <t>ng/ul</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/UO_0010050</t>
+  </si>
+  <si>
+    <t>pg/ul</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000438</t>
+  </si>
+  <si>
+    <t>library_layout</t>
+  </si>
+  <si>
+    <t>paired-end</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/OBI_0000722</t>
+  </si>
+  <si>
+    <t>single-end</t>
+  </si>
+  <si>
+    <t>http://purl.obolibrary.org/obo/OBI_0002481</t>
+  </si>
+  <si>
+    <t>number_of_pcr_cycles_for_indexing</t>
+  </si>
+  <si>
+    <t>library_preparation_kit</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 16 rxn; PN 1000283</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000250</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 4 rxn; PN 1000285</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000251</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Single Cell 3' GEM, Library &amp; Gel Bead Kit v3, 4 rxns; PN 1000092</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000260</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium Spatial Gene Expression Slide and Reagent Kit, 4 slides, 16 reactions; PN 1000184</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000261</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium Spatial Gene Expression Slide and Reagent Kit, 1 slides, 4 reactions; PN 1000187</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000265</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Single Cell 3' Library &amp; Gel Bead Kit, 4 rxns; PN 120267</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000299</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium Spatial for FFPE Gene Expression Kit, Human Transcriptome, 1 slides, 4 reactions; PN 1000338</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000320</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Human Transcriptome, 6.5mm, 4 reactions; PN 1000520</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000321</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Human Transcriptome, 11 mm, 2 reactions; PN 1000522</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000322</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' GEM, Library &amp; Gel Bead Kit v3.1, 16 rxns; PN 1000121</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000334</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' HT Kit v3.1, 48 rxns; PN 1000348</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000335</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' HT Kit v3.1, 8 rxns; PN 1000370</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000336</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' Kit v3.1, 16 rxns; PN 1000268</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000337</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 3' Kit v3.1, 4 rxns; PN 1000269</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000338</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 5' Kit v2, 16 rxns; PN 1000263</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000339</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell 5' Kit v2, 4 rxns; PN 1000265</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000340</t>
+  </si>
+  <si>
+    <t>Parse Biosciences; Evercode WT v2 Kit, 48 rxns; PN ECW02030</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000341</t>
+  </si>
+  <si>
+    <t>Parse Biosciences; Evercode WT Mini v2 Kit, 12 rxns; PN ECW02010</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000342</t>
+  </si>
+  <si>
+    <t>Illumina; TruSeq Stranded mRNA Library Prep (48 samples); PN 20020594</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000343</t>
+  </si>
+  <si>
+    <t>Illumina; TruSeq Stranded mRNA Library Prep (96 samples); PN 20020595</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000344</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium Spatial for FFPE Gene Expression Kit, Mouse Transcriptome, 4 rxns; PN 1000339</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000355</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Automated Single Cell 5' Kit v2, 24 rxns; PN 1000290</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000365</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Automated Single Cell 5' Kit v2, 4 rxns; PN 1000298</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000366</t>
+  </si>
+  <si>
+    <t>10X Genomics; Automated Library Construction Kit, 24 rxns; PN 1000428</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000374</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Hybridization &amp; Library Kit, 4 rxns; PN 1000415</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000375</t>
+  </si>
+  <si>
+    <t>New England BioLabs; NEBNext Ultra II RNA Library Prep Kit for Illumina; PN E7770</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000377</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium GEM-X Single Cell 5' Kit v3, 16 rxns; PN 1000699</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000394</t>
+  </si>
+  <si>
+    <t>10x Genomics; Library Construction Kit C, 4 rxns; PN 1000689</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000398</t>
+  </si>
+  <si>
+    <t>10x Genomics; Library Construction Kit C, 16 rxns; PN 1000694</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000399</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium GEM-X Single Cell 3' Kit v4, 16 rxns; PN 1000691</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000400</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Mouse Transcriptome, 6.5mm, 4 rxns; PN 1000521</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000432</t>
+  </si>
+  <si>
+    <t>10x Genomics; Library Construction Kit, 16 rxns; PN 1000190</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000439</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Single Cell 3ʹ GEM, Library &amp; Gel Bead Kit v3, 16 rxns; PN 1000075</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000460</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell 5' HT Kit v2, 8 rxns; PN 1000374</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000466</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell 5' HT Kit v2, 48 rxns; PN 1000356</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000467</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Single Cell ATAC Library &amp; Gel Bead Kit, 16 rxns; PN 1000110</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000469</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell ATAC Library &amp; Gel Bead Kit, 16 rxns; PN 1000175</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000471</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell Fixed RNA Sample Preparation Kit, 16 rxns; PN 1000414</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000484</t>
+  </si>
+  <si>
+    <t>10x Genomics; GEM-X Flex GEM &amp; Library Kit, 4 rxns; PN 1000782</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000497</t>
+  </si>
+  <si>
+    <t>Epigenome Technologies; Multiplex Droplet Paired-Tag 16 Reaction Kit; PN MDP16101</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000499</t>
+  </si>
+  <si>
+    <t>Takara Bio; SMART-Seq Total RNA Library Prep with ZapR Depletion (with UMIs), 96 rxns; PN 634355</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000507</t>
+  </si>
+  <si>
+    <t>sample_indexing_kit</t>
+  </si>
+  <si>
+    <t>10X Genomics; Single Index Kit N, Set A (96 rxn); PN 1000212</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000252</t>
+  </si>
+  <si>
+    <t>10X Genomics; Dual Index Kit TT, Set A (96 rxn); PN 1000215</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000253</t>
+  </si>
+  <si>
+    <t>10X Genomics; Dual Index Kit TS, Set A; PN 1000251</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000282</t>
+  </si>
+  <si>
+    <t>Parse Biosciences; Fragmentation Reagents; PN WX100</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000345</t>
+  </si>
+  <si>
+    <t>Parse Biosciences; UDI Plate - WT; PN UDI1001</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000346</t>
+  </si>
+  <si>
+    <t>Illumina; TruSeq RNA Single Indexes Set A (12 Indexes, 48 Samples); PN 20020492</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000347</t>
+  </si>
+  <si>
+    <t>Illumina; TruSeq RNA Single Indexes Set B (12 Indexes, 48 Samples); PN 20020493</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000348</t>
+  </si>
+  <si>
+    <t>Illumina; TruSeq RNA CD Index Plate (96 Indexes, 96 Samples); PN 20019792</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000349</t>
+  </si>
+  <si>
+    <t>Illumina; IDT for Illumina - TruSeq RNA UD Indexes v2 (96 Indexes, 96 Samples); PN 20040871</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000350</t>
+  </si>
+  <si>
+    <t>Integrated DNA Technologies: Custom DNA Oligos</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000351</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Seq Code Pack; PN GMX-NGS-SEQ-AB</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000356</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Seq Code Pack; PN GMX-NGS-SEQ-CD</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000357</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Seq Code Pack; PN GMX-NGS-SEQ-EF</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000358</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Seq Code Pack; PN GMX-NGS-SEQ-GH</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000359</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium i7 Sample Index Plate (96 rxn); PN 220103</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000380</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium i7 Multiplex Kit, 96 rxns; PN 120262</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000461</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium i7 Multiplex Kit N, Set A, 96 rxn; PN 1000084</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000468</t>
+  </si>
+  <si>
+    <t>Illumina; IDT for Illumina - TruSeq RNA UD Indexes (96 Indexes, 96 Samples); PN 20022371</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000505</t>
+  </si>
+  <si>
+    <t>Takara Bio; Unique Dual Index Kit (1–96), 96 rxns; PN 634752</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000508</t>
+  </si>
+  <si>
+    <t>Takara Bio; Unique Dual Index Kit (97–192), 96 rxns; PN 634753</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000509</t>
+  </si>
+  <si>
+    <t>Takara Bio; Unique Dual Index Kit (193–288), 96 rxns; PN 634754</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000510</t>
+  </si>
+  <si>
+    <t>Takara Bio; Unique Dual Index Kit (289–384), 96 rxns; PN 634755</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000511</t>
+  </si>
+  <si>
+    <t>Takara Bio; Unique Dual Index Kit (1–24), 24 rxns; PN 634756</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000512</t>
+  </si>
+  <si>
+    <t>sample_indexing_set</t>
+  </si>
+  <si>
+    <t>is_technical_replicate</t>
+  </si>
+  <si>
+    <t>sequencing_reagent_kit</t>
+  </si>
+  <si>
+    <t>Illumina; HiSeq 3000/4000 PE Cluster Kit PE-410-1001; PN 1000283</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000254</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 500/550 Hi Output Kit 150 Cycles; v2.5; PN 20024907</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000255</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 SP Reagent v1.5 Kit (100 Cycles); PN 20028401</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000256</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 S1 Reagent v1.5 Kit (100 Cycles); PN 20028319</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000257</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 S2 Reagent v1.5 Kit (100 Cycles); PN 20028316</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000258</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 S4 Reagent v1.5 Kit (200 Cycles); PN 20028313</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000259</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 10B Reagent Kit (300 Cycle); PN 20085594</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000283</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 10B Reagent Kit (200 Cycle); PN 20085595</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000284</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 10B Reagent Kit (100 Cycle); PN 20085596</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000285</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 1.5B Reagent Kit (100 Cycle); PN 20104703</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000286</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 1.5B Reagent Kit (200 Cycle); PN 20104704</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000287</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 1.5B Reagent Kit (300 Cycle); PN 20104705</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000288</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 S1 Reagent Kit (200 Cycles); PN 20012864</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000313</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 S1 Reagent v1.5 Kit (300 Cycles); PN 20028317</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000318</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 S4 Reagent Kit v1.5 (300 cycles); PN 20028312</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000319</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 1000/2000 P2 Reagent v3 Kit (100 Cycles); PN 20046811</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000323</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 1000/2000 P2 Reagent v3 Kit (200 Cycles); PN 20046812</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000352</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 1000/2000 P2 Reagent v3 Kit (300 Cycles); PN 20046813</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000353</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 2000 P3 Reagent Kit (300 Cycles); PN 20040561</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000354</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 S1 Reagent v1.5 Kit (200 Cycles); PN 20028318</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000360</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 2000 P3 Reagents Kit (100 Cycles); PN 20040559</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000361</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 500/550 Mid Output Kit 150 Cycles v2.5; PN 20024904</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000369</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 500/550 Hi Output Kit 75 Cycles v2.5; PN 20024906</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000381</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 25B Reagent Kit (300 Cycle); PN 20104706</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000392</t>
+  </si>
+  <si>
+    <t>Element Biosciences; AVITI 2x75 Sequencing Kit Cloudbreak FS High Output (184 Cycles); PN 860-00015</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000406</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq 6000 SP Reagent v1.5 Kit (300 Cycles); PN 20028400</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000459</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 25B Reagent Kit (100 Cycle); PN 20125967</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000463</t>
+  </si>
+  <si>
+    <t>Illumina; NovaSeq X Series 25B Reagent Kit (200 Cycle); PN 20125968</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000464</t>
+  </si>
+  <si>
+    <t>Illumina; NextSeq 1000/2000 P2 XLEAP-SBS Reagent Kit (100 Cycles); PN 20100987</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000503</t>
+  </si>
+  <si>
+    <t>Element Biosciences; AVITI 2x150 Sequencing Kit Cloudbreak FS High Output (334 Cycles); PN 860-00013</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000513</t>
+  </si>
+  <si>
+    <t>sequencing_read_format</t>
+  </si>
+  <si>
+    <t>sequencing_batch_id</t>
+  </si>
+  <si>
+    <t>preparation_instrument_vendor</t>
+  </si>
+  <si>
+    <t>HTX Technologies</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023734</t>
+  </si>
+  <si>
+    <t>SunChrom</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023908</t>
+  </si>
+  <si>
+    <t>Roche Diagnostics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025096</t>
+  </si>
+  <si>
+    <t>preparation_instrument_model</t>
+  </si>
+  <si>
+    <t>Chromium Controller</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_019326</t>
+  </si>
+  <si>
+    <t>Sublimator</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023729</t>
+  </si>
+  <si>
+    <t>M3+ Sprayer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023731</t>
+  </si>
+  <si>
+    <t>TM-Sprayer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023732</t>
+  </si>
+  <si>
+    <t>M5 Sprayer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023733</t>
+  </si>
+  <si>
+    <t>SunCollect Sprayer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023907</t>
+  </si>
+  <si>
+    <t>AutoStainer XL</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023957</t>
+  </si>
+  <si>
+    <t>Chromium iX</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024536</t>
+  </si>
+  <si>
+    <t>Chromium X</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024537</t>
+  </si>
+  <si>
+    <t>Visium CytAssist</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024570</t>
+  </si>
+  <si>
+    <t>ST5020 Multistainer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025021</t>
+  </si>
+  <si>
+    <t>Discovery Ultra</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025097</t>
+  </si>
+  <si>
+    <t>Chromium Connect</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025146</t>
+  </si>
+  <si>
+    <t>preparation_instrument_kit</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Chip J Single Cell Kit, 48 rxns; PN 1000234</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000262</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Chip J Single Cell Kit, 16 rxns; PN 1000230</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000263</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium FFPE Reagent Kit v2-Small, PN 1000436</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000324</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip Q Single Cell Kit, 16 rxns; PN 1000422</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000325</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip K Single Cell Kit, 48 rxns; PN 1000286</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000367</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip K Single Cell Kit, 16 rxns; PN 1000287</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000368</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip K Automated Single Cell Kit, 48 rxns; PN 1000289</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000373</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip G Single Cell Kit, 48 rxns; PN 1000120</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000378</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip G Single Cell Kit, 16 rxns; PN 1000127</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000379</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Single Cell B Chip Kit, 16 rxns; PN 1000074</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000462</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Chip E Single Cell ATAC Kit, 48 rxns; PN 1000155</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000470</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium HD, Human Transcriptome, 6.5 mm, 4 runs; PN 1000675</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000493</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium HD, Mouse Transcriptome, 6.5 mm, 4 runs; PN 1000676</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000494</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium HD, Human Transcriptome, 11 mm, 4 runs; PN 1001037</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000495</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium HD, Mouse Transcriptome, 11 mm, 4 runs; PN 1001038</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000496</t>
+  </si>
+  <si>
+    <t>10x Genomics; GEM-X Flex Gene Expression Chip Kit, 4 chips; PN 1000791</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000498</t>
+  </si>
+  <si>
+    <t>probe_hybridization_time_value</t>
+  </si>
+  <si>
+    <t>probe_hybridization_time_unit</t>
+  </si>
+  <si>
+    <t>oligo_probe_panel</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Human Transcriptome Probe Kit v2 - Small; PN 1000466</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000274</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Fixed RNA Kit, Human Transcriptome, 4 rxns x 1 BC; PN 1000474</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000306</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Human Transcriptome Probe Kit-Small; PN 1000363</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000326</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Mouse Transcriptome Probe Kit - Small; PN 1000365</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000362</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Human Whole Transcriptome Atlas, 4 slides; PN GMX-RNA-NGS-HuWTA-4</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000363</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Mouse Whole Transcriptome Atlas, 4 slides; PN GMX-RNA-NGS-MsWTA-4</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000364</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Human Transcriptome Probe Kit, 64 rxns; PN 1000456</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000376</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Human Transcriptome Probe Kit, 16 rxns; PN 1000420</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000382</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Human Transcriptome Probe Kit-Large; PN 1000364</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000383</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Single Cell Fixed RNA Mouse Transcriptome Probe Kit, 64 rxns; PN 1000492</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000393</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Human Multi-Tissue and Cancer Panel v1; PN 1000626</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000395</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Prime 5K Human Pan Tissue &amp; Pathways Panel; PN 1000724</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000426</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Human Universal Cell Characterization Panel (RNA, 1000 Plex); PN CMX-H-USCP-1KP-R</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000430</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium Mouse Transcriptome Probe Kit v2.0 - Small; PN 1000667</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000431</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Human Immuno-Oncology Panel (Protein, 64 Plex); PN CMX-H-IOP-64P-P</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000436</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Mouse Neuroscience Panel (Protein, 64 Plex); PN CMX-M-Neuro-64P-P</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000437</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Mouse Multi-Tissue Atlassing Panel; PN 1000627</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000442</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Human Lung Gene Expression Panel; PN 1000601</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000443</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Custom Gene Expression Panel (51-100 genes); PN 1000561</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000444</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Custom Gene Expression Panel (up to 50 genes); PN 1000464</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000445</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Human Colon Gene Expression Panel; PN 1000642</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000446</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Mouse Neuroscience Panel (RNA, 1000 Plex); PN CMX-M-NEUP-R</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000452</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Hs WTX RNA Panel Kit, 2 slides: PN 121500047</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000453</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Hs Univ Cell (RNA, 1000 Plex); PN 121500002</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000454</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Human 6K Discovery Panel (RNA, 6175 Plex); PN 121500041</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000455</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; CosMx Mouse Universal Cell Characterization Panel (RNA, 1000 Plex); PN CMX-M-USCP-1KP-R</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000457</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Fixed RNA Kit, Human Transcriptome 16 rxns x 16 BC; PN 1000547</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000477</t>
+  </si>
+  <si>
+    <t>10x Genomics; GEM-X Flex Human Transcriptome Probe Kit, 16 samples; PN 1000785</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000481</t>
+  </si>
+  <si>
+    <t>NanoString Technologies; GeoMx Human IO Proteome Atlas, 4 slides; PN 121300160</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000488</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Human Skin Gene Expression Panel; PN 1000643</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000491</t>
+  </si>
+  <si>
+    <t>10x Genomics; Xenium Prime 5K Mouse Pan Tissues &amp; Pathways Panel, 2 rxns; PN 1000725</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000506</t>
+  </si>
+  <si>
+    <t>is_custom_probes_used</t>
+  </si>
+  <si>
+    <t>metadata_schema_id</t>
+  </si>
+  <si>
+    <t>9a0570b7-b0ee-4e7e-a413-f95ae2f6cde7</t>
+  </si>
+  <si>
+    <t>schema:title</t>
+  </si>
+  <si>
     <t>Whole Exome Sequencing</t>
   </si>
   <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000514</t>
-  </si>
-  <si>
-    <t>analyte_class</t>
-  </si>
-  <si>
-    <t>Chromatin</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C13201</t>
-  </si>
-  <si>
-    <t>Collagen</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C16447</t>
-  </si>
-  <si>
-    <t>Protein</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17021</t>
-  </si>
-  <si>
-    <t>DNA</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C449</t>
-  </si>
-  <si>
-    <t>Metabolite</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C61154</t>
-  </si>
-  <si>
-    <t>Lipid</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C616</t>
-  </si>
-  <si>
-    <t>Peptide</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C735</t>
-  </si>
-  <si>
-    <t>RNA</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C812</t>
-  </si>
-  <si>
-    <t>Polysaccharide</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/CHEBI_18154</t>
-  </si>
-  <si>
-    <t>Fluorochrome</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/CHEBI_51217</t>
-  </si>
-  <si>
-    <t>Endogenous fluorophore</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000131</t>
-  </si>
-  <si>
-    <t>Nucleic acid + protein</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000273</t>
-  </si>
-  <si>
-    <t>DNA + RNA</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000327</t>
-  </si>
-  <si>
-    <t>Saturated lipid</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000388</t>
-  </si>
-  <si>
-    <t>Unsaturated lipid</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000389</t>
-  </si>
-  <si>
-    <t>Lipid + metabolite</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000401</t>
-  </si>
-  <si>
-    <t>RNA + protein</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000474</t>
-  </si>
-  <si>
-    <t>Lipid + metabolite + protein</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000478</t>
-  </si>
-  <si>
-    <t>is_targeted</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>acquisition_instrument_vendor</t>
-  </si>
-  <si>
-    <t>In-House</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C126386</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_003899</t>
-  </si>
-  <si>
-    <t>Thermo Fisher Scientific</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_008452</t>
-  </si>
-  <si>
-    <t>Leica Microsystems</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_008960</t>
-  </si>
-  <si>
-    <t>Miltenyi Biotec</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_008984</t>
-  </si>
-  <si>
-    <t>Illumina</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_010233</t>
-  </si>
-  <si>
-    <t>Hamamatsu</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_017105</t>
-  </si>
-  <si>
-    <t>Bruker</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_017365</t>
-  </si>
-  <si>
-    <t>Cytiva</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023581</t>
-  </si>
-  <si>
-    <t>Leica Biosystems</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023603</t>
-  </si>
-  <si>
-    <t>Keyence</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023604</t>
-  </si>
-  <si>
-    <t>Ionpath</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023605</t>
-  </si>
-  <si>
-    <t>Standard BioTools (Fluidigm)</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023606</t>
-  </si>
-  <si>
-    <t>Zeiss Microscopy</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023607</t>
-  </si>
-  <si>
-    <t>Andor</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023609</t>
-  </si>
-  <si>
-    <t>Sciex</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023651</t>
-  </si>
-  <si>
-    <t>10x Genomics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023672</t>
-  </si>
-  <si>
-    <t>Akoya Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023774</t>
-  </si>
-  <si>
-    <t>Resolve Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023911</t>
-  </si>
-  <si>
-    <t>NanoString</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023912</t>
-  </si>
-  <si>
-    <t>Waters</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024589</t>
-  </si>
-  <si>
-    <t>Evident Scientific (Olympus)</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024782</t>
-  </si>
-  <si>
-    <t>BGI Genomics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024848</t>
-  </si>
-  <si>
-    <t>Motic</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024856</t>
-  </si>
-  <si>
-    <t>Huron Digital Pathology</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024996</t>
-  </si>
-  <si>
-    <t>GE Healthcare</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025461</t>
-  </si>
-  <si>
-    <t>Vizgen</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026274</t>
-  </si>
-  <si>
-    <t>Element Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026453</t>
-  </si>
-  <si>
-    <t>Singular Genomics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026683</t>
-  </si>
-  <si>
-    <t>Complete Genomics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027007</t>
-  </si>
-  <si>
-    <t>3DHISTECH</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027042</t>
-  </si>
-  <si>
-    <t>Cytek Biosciences</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027071</t>
-  </si>
-  <si>
-    <t>Microscopes International</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027094</t>
-  </si>
-  <si>
-    <t>Revvity</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027779</t>
-  </si>
-  <si>
-    <t>MGI Tech</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_029020</t>
-  </si>
-  <si>
-    <t>acquisition_instrument_model</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C17998</t>
-  </si>
-  <si>
-    <t>Not applicable</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C48660</t>
-  </si>
-  <si>
-    <t>NextSeq 500</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_014983</t>
-  </si>
-  <si>
-    <t>NextSeq 550</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016381</t>
-  </si>
-  <si>
-    <t>HiSeq 2500</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016383</t>
-  </si>
-  <si>
-    <t>HiSeq 4000</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016386</t>
-  </si>
-  <si>
-    <t>NovaSeq 6000</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016387</t>
-  </si>
-  <si>
-    <t>iScan System</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_016388</t>
-  </si>
-  <si>
-    <t>BZ-X710</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_017202</t>
-  </si>
-  <si>
-    <t>LSM 710 Confocal Microscope</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_018063</t>
-  </si>
-  <si>
-    <t>Helios</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_019916</t>
-  </si>
-  <si>
-    <t>QTRAP 5500</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020517</t>
-  </si>
-  <si>
-    <t>Q Exactive HF</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020558</t>
-  </si>
-  <si>
-    <t>Orbitrap Fusion Tribrid</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020559</t>
-  </si>
-  <si>
-    <t>Orbitrap Fusion Lumos Tribrid</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020562</t>
-  </si>
-  <si>
-    <t>Q Exactive HF-X</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020564</t>
-  </si>
-  <si>
-    <t>Q Exactive</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020565</t>
-  </si>
-  <si>
-    <t>Q Exactive UHMR</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020571</t>
-  </si>
-  <si>
-    <t>Zeiss LightSheet Z.1</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020919</t>
-  </si>
-  <si>
-    <t>Axio Scan.Z1</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_020927</t>
-  </si>
-  <si>
-    <t>Aperio AT2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_021256</t>
-  </si>
-  <si>
-    <t>NanoZoomer 2.0-HT</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_021658</t>
-  </si>
-  <si>
-    <t>Digital Spatial Profiler</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_021660</t>
-  </si>
-  <si>
-    <t>Biomark HD</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_022658</t>
-  </si>
-  <si>
-    <t>Hyperion Imaging System</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023195</t>
-  </si>
-  <si>
-    <t>PhenoImager Fusion</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023274</t>
-  </si>
-  <si>
-    <t>Zyla 4.2 sCMOS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023610</t>
-  </si>
-  <si>
-    <t>SCN400</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023611</t>
-  </si>
-  <si>
-    <t>MIBIscope</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023613</t>
-  </si>
-  <si>
-    <t>NextSeq 2000</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023614</t>
-  </si>
-  <si>
-    <t>timsTOF FleX MALDI-2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023615</t>
-  </si>
-  <si>
-    <t>IN Cell Analyzer 2200</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023616</t>
-  </si>
-  <si>
-    <t>BZ-X800</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023617</t>
-  </si>
-  <si>
-    <t>Orbitrap Eclipse Tribrid</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023618</t>
-  </si>
-  <si>
-    <t>Axio Observer 5</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023692</t>
-  </si>
-  <si>
-    <t>Axio Observer 3</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023693</t>
-  </si>
-  <si>
-    <t>Axio Observer 7</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023694</t>
-  </si>
-  <si>
-    <t>NanoZoomer S210</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023760</t>
-  </si>
-  <si>
-    <t>NanoZoomer S360</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023761</t>
-  </si>
-  <si>
-    <t>NanoZoomer S60</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023762</t>
-  </si>
-  <si>
-    <t>NanoZoomer-SQ</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023763</t>
-  </si>
-  <si>
-    <t>Phenocycler-Fusion 2.0</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023773</t>
-  </si>
-  <si>
-    <t>CosMx Spatial Molecular Imager</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023909</t>
-  </si>
-  <si>
-    <t>Xenium Analyzer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023910</t>
-  </si>
-  <si>
-    <t>Lightsheet 7</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024448</t>
-  </si>
-  <si>
-    <t>Resolve Biosciences Molecular Cartography</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024449</t>
-  </si>
-  <si>
-    <t>NovaSeq X Plus</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024568</t>
-  </si>
-  <si>
-    <t>NovaSeq X</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024569</t>
-  </si>
-  <si>
-    <t>STELLARIS 5</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024663</t>
-  </si>
-  <si>
-    <t>VS200 Slide Scanner</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024783</t>
-  </si>
-  <si>
-    <t>Pannoramic MIDI II Digital Scanner</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024834</t>
-  </si>
-  <si>
-    <t>DNBSEQ-T7</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024847</t>
-  </si>
-  <si>
-    <t>MoticEasyScan One</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024855</t>
-  </si>
-  <si>
-    <t>DM6 B</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024857</t>
-  </si>
-  <si>
-    <t>TissueScope LE Slide Scanner</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024995</t>
-  </si>
-  <si>
-    <t>EVOS M7000</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025070</t>
-  </si>
-  <si>
-    <t>Aperio CS2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025111</t>
-  </si>
-  <si>
-    <t>BZ-X810</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025160</t>
-  </si>
-  <si>
-    <t>MERSCOPE Ultra</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026273</t>
-  </si>
-  <si>
-    <t>CyTOF XT</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026344</t>
-  </si>
-  <si>
-    <t>AVITI24</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026452</t>
-  </si>
-  <si>
-    <t>SYNAPT XS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026524</t>
-  </si>
-  <si>
-    <t>timsTOF Ultra</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026540</t>
-  </si>
-  <si>
-    <t>timsTOF Ultra 2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026541</t>
-  </si>
-  <si>
-    <t>timsTOF SCP</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026542</t>
-  </si>
-  <si>
-    <t>timsTOF HT</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026543</t>
-  </si>
-  <si>
-    <t>timsTOF Pro</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026544</t>
-  </si>
-  <si>
-    <t>timsTOF Pro 2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026545</t>
-  </si>
-  <si>
-    <t>CyTOF 2</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026551</t>
-  </si>
-  <si>
-    <t>DMi8</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026672</t>
-  </si>
-  <si>
-    <t>G4X Spatial Sequencer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026684</t>
-  </si>
-  <si>
-    <t>timsTOF FleX</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_026925</t>
-  </si>
-  <si>
-    <t>Cytek Northern Lights</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027072</t>
-  </si>
-  <si>
-    <t>Axio Zoom.V16</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027090</t>
-  </si>
-  <si>
-    <t>solariX</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027095</t>
-  </si>
-  <si>
-    <t>uScopeHXII-20</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027101</t>
-  </si>
-  <si>
-    <t>Juno System</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027198</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027323</t>
-  </si>
-  <si>
-    <t>Panoramic 150 Digital Scanner</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027467</t>
-  </si>
-  <si>
-    <t>Opera Phenix Plus HCS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027780</t>
-  </si>
-  <si>
-    <t>SYNAPT G2-Si</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027782</t>
-  </si>
-  <si>
-    <t>Opera Phenix HCS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027817</t>
-  </si>
-  <si>
-    <t>MACSima System</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_027923</t>
-  </si>
-  <si>
-    <t>NanoZoomer 2.0-RS</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_028001</t>
-  </si>
-  <si>
-    <t>Orbitrap Astral</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_028684</t>
-  </si>
-  <si>
-    <t>Olink Signature Q100</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_028906</t>
-  </si>
-  <si>
-    <t>Phenocycler-Fusion 1.0</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000316</t>
-  </si>
-  <si>
-    <t>Custom: Multiphoton</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000317</t>
-  </si>
-  <si>
-    <t>MERSCOPE</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000404</t>
-  </si>
-  <si>
-    <t>MALDI timsTOF Flex Prototype</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000433</t>
-  </si>
-  <si>
-    <t>source_storage_duration_value</t>
-  </si>
-  <si>
-    <t>source_storage_duration_unit</t>
-  </si>
-  <si>
-    <t>minute</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000031</t>
-  </si>
-  <si>
-    <t>hour</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000032</t>
-  </si>
-  <si>
-    <t>day</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000033</t>
-  </si>
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000035</t>
-  </si>
-  <si>
-    <t>year</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000036</t>
-  </si>
-  <si>
-    <t>time_since_acquisition_instrument_calibration_value</t>
-  </si>
-  <si>
-    <t>time_since_acquisition_instrument_calibration_unit</t>
-  </si>
-  <si>
-    <t>contributors_path</t>
-  </si>
-  <si>
-    <t>data_path</t>
-  </si>
-  <si>
-    <t>assay_input_entity</t>
-  </si>
-  <si>
-    <t>tissue (bulk)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000267</t>
-  </si>
-  <si>
-    <t>single cell</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000268</t>
-  </si>
-  <si>
-    <t>single nucleus</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000269</t>
-  </si>
-  <si>
-    <t>spot</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000270</t>
-  </si>
-  <si>
-    <t>area of interest</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000271</t>
-  </si>
-  <si>
-    <t>amount_of_input_analyte_value</t>
-  </si>
-  <si>
-    <t>amount_of_input_analyte_unit</t>
-  </si>
-  <si>
-    <t>ug</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000023</t>
-  </si>
-  <si>
-    <t>ng</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000024</t>
-  </si>
-  <si>
-    <t>library_adapter_sequence</t>
-  </si>
-  <si>
-    <t>library_average_fragment_size</t>
-  </si>
-  <si>
-    <t>dna_assay_input_value</t>
-  </si>
-  <si>
-    <t>dna_assay_input_unit</t>
-  </si>
-  <si>
-    <t>library_output_amount_value</t>
-  </si>
-  <si>
-    <t>library_output_amount_unit</t>
-  </si>
-  <si>
-    <t>ul</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000101</t>
-  </si>
-  <si>
-    <t>library_concentration_value</t>
-  </si>
-  <si>
-    <t>library_concentration_unit</t>
-  </si>
-  <si>
-    <t>nM</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0000065</t>
-  </si>
-  <si>
-    <t>ng/ul</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/UO_0010050</t>
-  </si>
-  <si>
-    <t>pg/ul</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000438</t>
-  </si>
-  <si>
-    <t>library_layout</t>
-  </si>
-  <si>
-    <t>paired-end</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/OBI_0000722</t>
-  </si>
-  <si>
-    <t>single-end</t>
-  </si>
-  <si>
-    <t>http://purl.obolibrary.org/obo/OBI_0002481</t>
-  </si>
-  <si>
-    <t>number_of_pcr_cycles_for_indexing</t>
-  </si>
-  <si>
-    <t>library_preparation_kit</t>
-  </si>
-  <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 16 rxn; PN 1000283</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000250</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 4 rxn; PN 1000285</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000251</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Single Cell 3' GEM, Library &amp; Gel Bead Kit v3, 4 rxns; PN 1000092</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000260</t>
-  </si>
-  <si>
-    <t>10X Genomics; Visium Spatial Gene Expression Slide and Reagent Kit, 4 slides, 16 reactions; PN 1000184</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000261</t>
-  </si>
-  <si>
-    <t>10X Genomics; Visium Spatial Gene Expression Slide and Reagent Kit, 1 slides, 4 reactions; PN 1000187</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000265</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Single Cell 3' Library &amp; Gel Bead Kit, 4 rxns; PN 120267</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000299</t>
-  </si>
-  <si>
-    <t>10X Genomics; Visium Spatial for FFPE Gene Expression Kit, Human Transcriptome, 1 slides, 4 reactions; PN 1000338</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000320</t>
-  </si>
-  <si>
-    <t>10X Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Human Transcriptome, 6.5mm, 4 reactions; PN 1000520</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000321</t>
-  </si>
-  <si>
-    <t>10X Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Human Transcriptome, 11 mm, 2 reactions; PN 1000522</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000322</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell 3' GEM, Library &amp; Gel Bead Kit v3.1, 16 rxns; PN 1000121</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000334</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell 3' HT Kit v3.1, 48 rxns; PN 1000348</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000335</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell 3' HT Kit v3.1, 8 rxns; PN 1000370</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000336</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell 3' Kit v3.1, 16 rxns; PN 1000268</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000337</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell 3' Kit v3.1, 4 rxns; PN 1000269</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000338</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell 5' Kit v2, 16 rxns; PN 1000263</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000339</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell 5' Kit v2, 4 rxns; PN 1000265</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000340</t>
-  </si>
-  <si>
-    <t>Parse Biosciences; Evercode WT v2 Kit, 48 rxns; PN ECW02030</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000341</t>
-  </si>
-  <si>
-    <t>Parse Biosciences; Evercode WT Mini v2 Kit, 12 rxns; PN ECW02010</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000342</t>
-  </si>
-  <si>
-    <t>Illumina; TruSeq Stranded mRNA Library Prep (48 samples); PN 20020594</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000343</t>
-  </si>
-  <si>
-    <t>Illumina; TruSeq Stranded mRNA Library Prep (96 samples); PN 20020595</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000344</t>
-  </si>
-  <si>
-    <t>10X Genomics; Visium Spatial for FFPE Gene Expression Kit, Mouse Transcriptome, 4 rxns; PN 1000339</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000355</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Automated Single Cell 5' Kit v2, 24 rxns; PN 1000290</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000365</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Automated Single Cell 5' Kit v2, 4 rxns; PN 1000298</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000366</t>
-  </si>
-  <si>
-    <t>10X Genomics; Automated Library Construction Kit, 24 rxns; PN 1000428</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000374</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Hybridization &amp; Library Kit, 4 rxns; PN 1000415</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000375</t>
-  </si>
-  <si>
-    <t>New England BioLabs; NEBNext Ultra II RNA Library Prep Kit for Illumina; PN E7770</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000377</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium GEM-X Single Cell 5' Kit v3, 16 rxns; PN 1000699</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000394</t>
-  </si>
-  <si>
-    <t>10x Genomics; Library Construction Kit C, 4 rxns; PN 1000689</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000398</t>
-  </si>
-  <si>
-    <t>10x Genomics; Library Construction Kit C, 16 rxns; PN 1000694</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000399</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium GEM-X Single Cell 3' Kit v4, 16 rxns; PN 1000691</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000400</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium CytAssist Spatial Gene Expression for FFPE, Mouse Transcriptome, 6.5mm, 4 rxns; PN 1000521</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000432</t>
-  </si>
-  <si>
-    <t>10x Genomics; Library Construction Kit, 16 rxns; PN 1000190</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000439</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Single Cell 3ʹ GEM, Library &amp; Gel Bead Kit v3, 16 rxns; PN 1000075</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000460</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Next GEM Single Cell 5' HT Kit v2, 8 rxns; PN 1000374</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000466</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Next GEM Single Cell 5' HT Kit v2, 48 rxns; PN 1000356</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000467</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Single Cell ATAC Library &amp; Gel Bead Kit, 16 rxns; PN 1000110</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000469</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Next GEM Single Cell ATAC Library &amp; Gel Bead Kit, 16 rxns; PN 1000175</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000471</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Next GEM Single Cell Fixed RNA Sample Preparation Kit, 16 rxns; PN 1000414</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000484</t>
-  </si>
-  <si>
-    <t>10x Genomics; GEM-X Flex GEM &amp; Library Kit, 4 rxns; PN 1000782</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000497</t>
-  </si>
-  <si>
-    <t>Epigenome Technologies; Multiplex Droplet Paired-Tag 16 Reaction Kit; PN MDP16101</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000499</t>
-  </si>
-  <si>
-    <t>Takara Bio; SMART-Seq Total RNA Library Prep with ZapR Depletion (with UMIs), 96 rxns; PN 634355</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000507</t>
-  </si>
-  <si>
-    <t>sample_indexing_kit</t>
-  </si>
-  <si>
-    <t>10X Genomics; Single Index Kit N, Set A (96 rxn); PN 1000212</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000252</t>
-  </si>
-  <si>
-    <t>10X Genomics; Dual Index Kit TT, Set A (96 rxn); PN 1000215</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000253</t>
-  </si>
-  <si>
-    <t>10X Genomics; Dual Index Kit TS, Set A; PN 1000251</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000282</t>
-  </si>
-  <si>
-    <t>Parse Biosciences; Fragmentation Reagents; PN WX100</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000345</t>
-  </si>
-  <si>
-    <t>Parse Biosciences; UDI Plate - WT; PN UDI1001</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000346</t>
-  </si>
-  <si>
-    <t>Illumina; TruSeq RNA Single Indexes Set A (12 Indexes, 48 Samples); PN 20020492</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000347</t>
-  </si>
-  <si>
-    <t>Illumina; TruSeq RNA Single Indexes Set B (12 Indexes, 48 Samples); PN 20020493</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000348</t>
-  </si>
-  <si>
-    <t>Illumina; TruSeq RNA CD Index Plate (96 Indexes, 96 Samples); PN 20019792</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000349</t>
-  </si>
-  <si>
-    <t>Illumina; IDT for Illumina - TruSeq RNA UD Indexes v2 (96 Indexes, 96 Samples); PN 20040871</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000350</t>
-  </si>
-  <si>
-    <t>Integrated DNA Technologies: Custom DNA Oligos</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000351</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Seq Code Pack; PN GMX-NGS-SEQ-AB</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000356</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Seq Code Pack; PN GMX-NGS-SEQ-CD</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000357</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Seq Code Pack; PN GMX-NGS-SEQ-EF</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000358</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Seq Code Pack; PN GMX-NGS-SEQ-GH</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000359</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium i7 Sample Index Plate (96 rxn); PN 220103</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000380</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium i7 Multiplex Kit, 96 rxns; PN 120262</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000461</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium i7 Multiplex Kit N, Set A, 96 rxn; PN 1000084</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000468</t>
-  </si>
-  <si>
-    <t>Illumina; IDT for Illumina - TruSeq RNA UD Indexes (96 Indexes, 96 Samples); PN 20022371</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000505</t>
-  </si>
-  <si>
-    <t>Takara Bio; Unique Dual Index Kit (1–96), 96 rxns; PN 634752</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000508</t>
-  </si>
-  <si>
-    <t>Takara Bio; Unique Dual Index Kit (97–192), 96 rxns; PN 634753</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000509</t>
-  </si>
-  <si>
-    <t>Takara Bio; Unique Dual Index Kit (193–288), 96 rxns; PN 634754</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000510</t>
-  </si>
-  <si>
-    <t>Takara Bio; Unique Dual Index Kit (289–384), 96 rxns; PN 634755</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000511</t>
-  </si>
-  <si>
-    <t>Takara Bio; Unique Dual Index Kit (1–24), 24 rxns; PN 634756</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000512</t>
-  </si>
-  <si>
-    <t>sample_indexing_set</t>
-  </si>
-  <si>
-    <t>is_technical_replicate</t>
-  </si>
-  <si>
-    <t>sequencing_reagent_kit</t>
-  </si>
-  <si>
-    <t>Illumina; HiSeq 3000/4000 PE Cluster Kit PE-410-1001; PN 1000283</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000254</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 500/550 Hi Output Kit 150 Cycles; v2.5; PN 20024907</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000255</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 SP Reagent v1.5 Kit (100 Cycles); PN 20028401</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000256</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 S1 Reagent v1.5 Kit (100 Cycles); PN 20028319</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000257</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 S2 Reagent v1.5 Kit (100 Cycles); PN 20028316</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000258</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 S4 Reagent v1.5 Kit (200 Cycles); PN 20028313</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000259</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 10B Reagent Kit (300 Cycle); PN 20085594</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000283</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 10B Reagent Kit (200 Cycle); PN 20085595</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000284</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 10B Reagent Kit (100 Cycle); PN 20085596</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000285</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 1.5B Reagent Kit (100 Cycle); PN 20104703</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000286</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 1.5B Reagent Kit (200 Cycle); PN 20104704</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000287</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 1.5B Reagent Kit (300 Cycle); PN 20104705</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000288</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 S1 Reagent Kit (200 Cycles); PN 20012864</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000313</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 S1 Reagent v1.5 Kit (300 Cycles); PN 20028317</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000318</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 S4 Reagent Kit v1.5 (300 cycles); PN 20028312</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000319</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 1000/2000 P2 Reagent v3 Kit (100 Cycles); PN 20046811</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000323</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 1000/2000 P2 Reagent v3 Kit (200 Cycles); PN 20046812</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000352</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 1000/2000 P2 Reagent v3 Kit (300 Cycles); PN 20046813</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000353</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 2000 P3 Reagent Kit (300 Cycles); PN 20040561</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000354</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 S1 Reagent v1.5 Kit (200 Cycles); PN 20028318</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000360</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 2000 P3 Reagents Kit (100 Cycles); PN 20040559</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000361</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 500/550 Mid Output Kit 150 Cycles v2.5; PN 20024904</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000369</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 500/550 Hi Output Kit 75 Cycles v2.5; PN 20024906</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000381</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 25B Reagent Kit (300 Cycle); PN 20104706</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000392</t>
-  </si>
-  <si>
-    <t>Element Biosciences; AVITI 2x75 Sequencing Kit Cloudbreak FS High Output (184 Cycles); PN 860-00015</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000406</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq 6000 SP Reagent v1.5 Kit (300 Cycles); PN 20028400</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000459</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 25B Reagent Kit (100 Cycle); PN 20125967</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000463</t>
-  </si>
-  <si>
-    <t>Illumina; NovaSeq X Series 25B Reagent Kit (200 Cycle); PN 20125968</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000464</t>
-  </si>
-  <si>
-    <t>Illumina; NextSeq 1000/2000 P2 XLEAP-SBS Reagent Kit (100 Cycles); PN 20100987</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000503</t>
-  </si>
-  <si>
-    <t>Element Biosciences; AVITI 2x150 Sequencing Kit Cloudbreak FS High Output (334 Cycles); PN 860-00013</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000513</t>
-  </si>
-  <si>
-    <t>sequencing_read_format</t>
-  </si>
-  <si>
-    <t>sequencing_batch_id</t>
-  </si>
-  <si>
-    <t>preparation_instrument_vendor</t>
-  </si>
-  <si>
-    <t>HTX Technologies</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023734</t>
-  </si>
-  <si>
-    <t>SunChrom</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023908</t>
-  </si>
-  <si>
-    <t>Roche Diagnostics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025096</t>
-  </si>
-  <si>
-    <t>preparation_instrument_model</t>
-  </si>
-  <si>
-    <t>Chromium Controller</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_019326</t>
-  </si>
-  <si>
-    <t>Sublimator</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023729</t>
-  </si>
-  <si>
-    <t>M3+ Sprayer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023731</t>
-  </si>
-  <si>
-    <t>TM-Sprayer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023732</t>
-  </si>
-  <si>
-    <t>M5 Sprayer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023733</t>
-  </si>
-  <si>
-    <t>SunCollect Sprayer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023907</t>
-  </si>
-  <si>
-    <t>AutoStainer XL</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023957</t>
-  </si>
-  <si>
-    <t>Chromium iX</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024536</t>
-  </si>
-  <si>
-    <t>Chromium X</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024537</t>
-  </si>
-  <si>
-    <t>Visium CytAssist</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024570</t>
-  </si>
-  <si>
-    <t>ST5020 Multistainer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025021</t>
-  </si>
-  <si>
-    <t>Discovery Ultra</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025097</t>
-  </si>
-  <si>
-    <t>Chromium Connect</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025146</t>
-  </si>
-  <si>
-    <t>preparation_instrument_kit</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Next GEM Chip J Single Cell Kit, 48 rxns; PN 1000234</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000262</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Next GEM Chip J Single Cell Kit, 16 rxns; PN 1000230</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000263</t>
-  </si>
-  <si>
-    <t>10X Genomics; Visium FFPE Reagent Kit v2-Small, PN 1000436</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000324</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip Q Single Cell Kit, 16 rxns; PN 1000422</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000325</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip K Single Cell Kit, 48 rxns; PN 1000286</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000367</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip K Single Cell Kit, 16 rxns; PN 1000287</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000368</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip K Automated Single Cell Kit, 48 rxns; PN 1000289</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000373</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip G Single Cell Kit, 48 rxns; PN 1000120</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000378</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip G Single Cell Kit, 16 rxns; PN 1000127</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000379</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Single Cell B Chip Kit, 16 rxns; PN 1000074</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000462</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Chip E Single Cell ATAC Kit, 48 rxns; PN 1000155</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000470</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium HD, Human Transcriptome, 6.5 mm, 4 runs; PN 1000675</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000493</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium HD, Mouse Transcriptome, 6.5 mm, 4 runs; PN 1000676</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000494</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium HD, Human Transcriptome, 11 mm, 4 runs; PN 1001037</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000495</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium HD, Mouse Transcriptome, 11 mm, 4 runs; PN 1001038</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000496</t>
-  </si>
-  <si>
-    <t>10x Genomics; GEM-X Flex Gene Expression Chip Kit, 4 chips; PN 1000791</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000498</t>
-  </si>
-  <si>
-    <t>probe_hybridization_time_value</t>
-  </si>
-  <si>
-    <t>probe_hybridization_time_unit</t>
-  </si>
-  <si>
-    <t>oligo_probe_panel</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium Human Transcriptome Probe Kit v2 - Small; PN 1000466</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000274</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Fixed RNA Kit, Human Transcriptome, 4 rxns x 1 BC; PN 1000474</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000306</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium Human Transcriptome Probe Kit-Small; PN 1000363</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000326</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium Mouse Transcriptome Probe Kit - Small; PN 1000365</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000362</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Human Whole Transcriptome Atlas, 4 slides; PN GMX-RNA-NGS-HuWTA-4</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000363</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Mouse Whole Transcriptome Atlas, 4 slides; PN GMX-RNA-NGS-MsWTA-4</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000364</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Human Transcriptome Probe Kit, 64 rxns; PN 1000456</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000376</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Single Cell Fixed RNA Human Transcriptome Probe Kit, 16 rxns; PN 1000420</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000382</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium Human Transcriptome Probe Kit-Large; PN 1000364</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000383</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Next GEM Single Cell Fixed RNA Mouse Transcriptome Probe Kit, 64 rxns; PN 1000492</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000393</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Human Multi-Tissue and Cancer Panel v1; PN 1000626</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000395</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Prime 5K Human Pan Tissue &amp; Pathways Panel; PN 1000724</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000426</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Human Universal Cell Characterization Panel (RNA, 1000 Plex); PN CMX-H-USCP-1KP-R</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000430</t>
-  </si>
-  <si>
-    <t>10x Genomics; Visium Mouse Transcriptome Probe Kit v2.0 - Small; PN 1000667</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000431</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Human Immuno-Oncology Panel (Protein, 64 Plex); PN CMX-H-IOP-64P-P</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000436</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Mouse Neuroscience Panel (Protein, 64 Plex); PN CMX-M-Neuro-64P-P</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000437</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Mouse Multi-Tissue Atlassing Panel; PN 1000627</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000442</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Human Lung Gene Expression Panel; PN 1000601</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000443</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Custom Gene Expression Panel (51-100 genes); PN 1000561</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000444</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Custom Gene Expression Panel (up to 50 genes); PN 1000464</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000445</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Human Colon Gene Expression Panel; PN 1000642</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000446</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Mouse Neuroscience Panel (RNA, 1000 Plex); PN CMX-M-NEUP-R</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000452</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Hs WTX RNA Panel Kit, 2 slides: PN 121500047</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000453</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Hs Univ Cell (RNA, 1000 Plex); PN 121500002</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000454</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Human 6K Discovery Panel (RNA, 6175 Plex); PN 121500041</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000455</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; CosMx Mouse Universal Cell Characterization Panel (RNA, 1000 Plex); PN CMX-M-USCP-1KP-R</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000457</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium Fixed RNA Kit, Human Transcriptome 16 rxns x 16 BC; PN 1000547</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000477</t>
-  </si>
-  <si>
-    <t>10x Genomics; GEM-X Flex Human Transcriptome Probe Kit, 16 samples; PN 1000785</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000481</t>
-  </si>
-  <si>
-    <t>NanoString Technologies; GeoMx Human IO Proteome Atlas, 4 slides; PN 121300160</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000488</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Human Skin Gene Expression Panel; PN 1000643</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000491</t>
-  </si>
-  <si>
-    <t>10x Genomics; Xenium Prime 5K Mouse Pan Tissues &amp; Pathways Panel, 2 rxns; PN 1000725</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000506</t>
-  </si>
-  <si>
-    <t>is_custom_probes_used</t>
-  </si>
-  <si>
-    <t>metadata_schema_id</t>
-  </si>
-  <si>
-    <t>9a0570b7-b0ee-4e7e-a413-f95ae2f6cde7</t>
-  </si>
-  <si>
-    <t>schema:title</t>
-  </si>
-  <si>
     <t>pav:version</t>
   </si>
   <si>
@@ -2778,7 +2781,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2026-10-22T09:20:24-07:00</t>
+    <t>2026-10-23T08:05:59-07:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -5403,27 +5406,27 @@
         <v>801</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>806</v>
+        <v>807</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>122</v>
+        <v>802</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>807</v>
+        <v>808</v>
       </c>
     </row>
   </sheetData>

</xml_diff>